<commit_message>
feat(multas): preservar multas históricas de estudiantes inactivos
</commit_message>
<xml_diff>
--- a/Frontend/public/plantillas/plantilla-carga-masiva-multas.xlsx
+++ b/Frontend/public/plantillas/plantilla-carga-masiva-multas.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multas" sheetId="1" r:id="Rf361ac4579274518"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rc165a08b914244c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multas" sheetId="1" r:id="R230d1b4d8513463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R48b29800122d4502"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +24,7 @@
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="10"/>
+      <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
@@ -60,7 +60,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF252A34"/>
+        <x:fgColor rgb="FFF4D6DC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -82,16 +82,16 @@
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD1D5DB"/>
+        <x:color rgb="FFD6DAE1"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFD1D5DB"/>
+        <x:color rgb="FFD6DAE1"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFD1D5DB"/>
+        <x:color rgb="FFD6DAE1"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFD1D5DB"/>
+        <x:color rgb="FFD6DAE1"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -112,29 +112,29 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -144,6 +144,31 @@
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlantillaMultas" displayName="PlantillaMultas" ref="A1:F2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Estudiante"/>
+    <x:tableColumn id="2" name="Motivo"/>
+    <x:tableColumn id="3" name="Fecha"/>
+    <x:tableColumn id="4" name="Descripción"/>
+    <x:tableColumn id="5" name="Multa sugerida"/>
+    <x:tableColumn id="6" name="Estado"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="InstruccionesMultas" displayName="InstruccionesMultas" ref="A3:C9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="Campo"/>
+    <x:tableColumn id="2" name="Formato"/>
+    <x:tableColumn id="3" name="Ejemplo"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -341,61 +366,64 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Multa</x:v>
+        <x:v>Estudiante</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>Estudiante</x:v>
+        <x:v>Motivo</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
-        <x:v>Motivo</x:v>
+        <x:v>Fecha</x:v>
       </x:c>
       <x:c r="D1" s="5" t="str">
-        <x:v>Fecha</x:v>
+        <x:v>Descripción</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>Descripción</x:v>
+        <x:v>Multa sugerida</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>Multa sugerida</x:v>
-      </x:c>
-      <x:c r="G1" s="5" t="str">
         <x:v>Estado</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="44" customHeight="1">
-      <x:c r="A2" s="9" t="str"/>
-      <x:c r="B2" s="9" t="str">
+    <x:row r="2" ht="48" customHeight="1">
+      <x:c r="A2" s="8" t="str">
         <x:v>20261001 - NOMBRE COMPLETO DEL ESTUDIANTE</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str">
+      <x:c r="B2" s="8" t="str">
         <x:v>Incumplimiento de la devolución</x:v>
       </x:c>
-      <x:c r="D2" s="10" t="n">
+      <x:c r="C2" s="9" t="n">
         <x:v>46274</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="str">
+      <x:c r="D2" s="8" t="str">
         <x:v>Describa brevemente la situación que originó la multa.</x:v>
       </x:c>
-      <x:c r="F2" s="9" t="str">
+      <x:c r="E2" s="8" t="str">
         <x:v>Indique el compromiso o acción sugerida.</x:v>
       </x:c>
-      <x:c r="G2" s="9" t="str">
+      <x:c r="F2" s="8" t="str">
         <x:v>ACTIVA</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="F2:F5001">
+      <x:formula1>"ACTIVA,CUMPLIDA,ANULADA"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R311a91677dca4077"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -403,103 +431,97 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="19" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="68" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="13" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="11" t="str">
         <x:v>Carga masiva de multas</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str"/>
-      <x:c r="C1" s="13" t="str"/>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="18" t="str">
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="16" t="str">
         <x:v>Campo</x:v>
       </x:c>
-      <x:c r="B3" s="18" t="str">
+      <x:c r="B3" s="16" t="str">
         <x:v>Formato</x:v>
       </x:c>
-      <x:c r="C3" s="18" t="str">
+      <x:c r="C3" s="16" t="str">
         <x:v>Ejemplo</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="42" customHeight="1">
+    <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="19" t="str">
-        <x:v>Multa</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>Opcional. Déjelo vacío para crear una multa. Use el folio existente para actualizarla.</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>MUL-ABC12345</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="42" customHeight="1">
+        <x:v>Estudiante</x:v>
+      </x:c>
+      <x:c r="B4" s="18" t="str">
+        <x:v>Obligatorio. Debe iniciar con el código numérico, seguido de un guion y el nombre.</x:v>
+      </x:c>
+      <x:c r="C4" s="18" t="str">
+        <x:v>20261001 - NOMBRE COMPLETO DEL ESTUDIANTE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
       <x:c r="A5" s="19" t="str">
-        <x:v>Estudiante</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>Obligatorio. Debe iniciar con el código numérico, seguido de un guion y el nombre.</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>20261001 - NOMBRE COMPLETO DEL ESTUDIANTE</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="42" customHeight="1">
+        <x:v>Motivo</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="str">
+        <x:v>Obligatorio. Se crea o reutiliza automáticamente según el nombre.</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="str">
+        <x:v>Incumplimiento de la devolución</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="19" t="str">
-        <x:v>Motivo</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>Obligatorio. Se crea o reutiliza automáticamente según el nombre.</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>Incumplimiento de la devolución</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
+        <x:v>Fecha</x:v>
+      </x:c>
+      <x:c r="B6" s="18" t="str">
+        <x:v>Obligatoria. Use el formato AAAA-MM-DD.</x:v>
+      </x:c>
+      <x:c r="C6" s="18" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="19" t="str">
-        <x:v>Fecha</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Obligatoria. Use el formato AAAA-MM-DD.</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
+        <x:v>Descripción</x:v>
+      </x:c>
+      <x:c r="B7" s="18" t="str">
+        <x:v>Obligatoria. Explique brevemente la situación.</x:v>
+      </x:c>
+      <x:c r="C7" s="18" t="str">
+        <x:v>No realizó la devolución en el horario acordado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="19" t="str">
-        <x:v>Descripción</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>Obligatoria. Explique brevemente la situación.</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>No realizó la devolución en el horario acordado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
+        <x:v>Multa sugerida</x:v>
+      </x:c>
+      <x:c r="B8" s="18" t="str">
+        <x:v>Opcional. Registre el compromiso o acción sugerida.</x:v>
+      </x:c>
+      <x:c r="C8" s="18" t="str">
+        <x:v>Devolver los elementos pendientes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
       <x:c r="A9" s="19" t="str">
-        <x:v>Multa sugerida</x:v>
-      </x:c>
-      <x:c r="B9" s="9" t="str">
-        <x:v>Opcional. Registre el compromiso o acción sugerida.</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>Devolver los elementos pendientes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="19" t="str">
         <x:v>Estado</x:v>
       </x:c>
-      <x:c r="B10" s="9" t="str">
+      <x:c r="B9" s="18" t="str">
         <x:v>Obligatorio. Solo se acepta ACTIVA, CUMPLIDA o ANULADA.</x:v>
       </x:c>
-      <x:c r="C10" s="9" t="str">
+      <x:c r="C9" s="18" t="str">
         <x:v>ACTIVA</x:v>
       </x:c>
     </x:row>
@@ -508,5 +530,8 @@
     <x:mergeCell ref="A1:C1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raac6f8b03c5f47c7"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>